<commit_message>
feat: gemini 오류 수정
</commit_message>
<xml_diff>
--- a/data/market_excel/market_final_네패스.xlsx
+++ b/data/market_excel/market_final_네패스.xlsx
@@ -530,29 +530,13 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>네패스는 AI 시대의 핵심인 반도체 후공정/패키징 분야에서 높은 성장 잠재력을 가지고 있습니다. 최근 주가 모멘텀도 긍정적이나, 거시 경제 불확실성과 높은 경쟁 강도가 리스크 요인으로 작용합니다. 따라서 '보유' 의견을 제시합니다.</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>후공정/패키징/테스트</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
+          <t>네패스는 AI 시대의 핵심인 반도체 후공정/패키징 분야에서 높은 성장 잠재력을 보유하고 있습니다. 최근 주가 모멘텀은 긍정적이나, 거시 경제 불확실성과 경쟁 심화가 리스크 요인으로 작용합니다. 따라서 '보유' 의견을 제시합니다.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -646,7 +630,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>네패스는 AI 시대의 핵심인 반도체 후공정/패키징 분야에서 높은 성장 잠재력을 가지고 있습니다. 최근 주가 모멘텀도 긍정적이나, 거시 경제 불확실성과 높은 경쟁 강도가 리스크 요인으로 작용합니다. 따라서 '보유' 의견을 제시합니다.</t>
+          <t>네패스는 AI 시대의 핵심인 반도체 후공정/패키징 분야에서 높은 성장 잠재력을 보유하고 있습니다. 최근 주가 모멘텀은 긍정적이나, 거시 경제 불확실성과 경쟁 심화가 리스크 요인으로 작용합니다. 따라서 '보유' 의견을 제시합니다.</t>
         </is>
       </c>
     </row>
@@ -742,20 +726,16 @@
           <t>N</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>한미반도체, ISC, SFA반도체, 두산테스나, 리노공업</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>높음</t>
+          <t>중간</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>네패스는 첨단 후공정 파운드리 사업과 반도체/디스플레이 제조에 사용되는 전자재료사업을 통해 스마트폰 및 다양한 전자기기에 필수적인 기술을 제공합니다.</t>
+          <t>세계 유수의 반도체 업체들에게 최첨단 반도체 패키징 솔루션을 제공하여 업계에서 신뢰받는 기업으로 자리 잡고 있습니다.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -765,22 +745,22 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>사업보고서에서 반도체의 후공정 파운드리 사업과 전자재료사업이 언급되었기 때문에 후공정/패키징/테스트로 분류하였습니다.</t>
+          <t>사업 개요에서 반도체 조립 및 테스트 제품을 주력으로 생산하고 있다고 명시되어 있습니다.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>네패스</t>
+          <t>SFA반도체</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>20241114002980</t>
+          <t>20241113000459</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-05-25T00:27:03.901541</t>
+          <t>2026-05-25T11:09:12.756789</t>
         </is>
       </c>
     </row>

</xml_diff>